<commit_message>
Leads: 2026-10-13 02:00 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,6 @@
           <t>https://fixmyairandheat.com/locations/air-conditioning-repair-fontana-ca/</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>service@relaxedheatingandair.com</t>
@@ -580,7 +579,6 @@
           <t>https://www.apexroofingsolutions.com/services/metal-roofing/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>john@smith.com</t>
@@ -610,6 +608,66 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lawrence Plumbing, LLC |</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>lawrenceplumbingomaha.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://lawrenceplumbingomaha.com/plumbing-services-la-vista-ne/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>La Vista</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>lawrenceplumbing.biz@gmail.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(402) 201-0709</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Bellevue NE</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>94</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>plumber Bellevue NE</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-13 02:02 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -673,6 +673,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OneSource Roofing &amp; Restoration | Premier DFW Roofing Services</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>onesourceroofs.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://onesourceroofs.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>If You</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>contact@onesourceroofs.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>972-928-2988</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>80</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roof replacement Frisco TX</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-13 02:11 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -733,6 +733,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AAA Crop</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>aaanycorp.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://aaanycorp.com/roofing-contractor-new-york/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Tanveer Ahmed</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>aaanycontractingcorp@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(914) 912-1067</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Bronx NY</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>residential roofing company Bronx NY</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-13 11:36 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -793,6 +793,126 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>My Water Heater Repair</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>mywaterheaterrepair.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://mywaterheaterrepair.com/maryland/rockville/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Testimonials What</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>service@mywaterheaterrepair.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>877 835 0417</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Rockville MD</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>88</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>water heater repair Rockville MD</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Maxx Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>maxxroofing.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://maxxroofing.com/roofing/broken-arrow/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Founded Family</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>office@maxxroofing.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(918) 893-9595</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>80</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>roof repair company Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-13 11:38 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -913,6 +913,62 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Superior Roofing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>superiorroofingks.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://superiorroofingks.com/residential/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>kansashomes1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(316) 516-0139</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>80</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>residential roofing company Wichita KS</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-13 11:40 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -934,7 +934,6 @@
           <t>https://superiorroofingks.com/residential/</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>kansashomes1@gmail.com</t>
@@ -964,6 +963,62 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Charlotte Water Heater Experts</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>charlottewaterheaterexperts.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://charlottewaterheaterexperts.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Charlotte Water</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>evershieldllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Charlotte NC</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>78</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>water heater repair Charlotte NC</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-13 11:41 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -999,7 +999,6 @@
           <t>evershieldllc@gmail.com</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Charlotte NC</t>
@@ -1019,6 +1018,66 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Corona</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>corona-ca.metalproroofingarcadia.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://corona-ca.metalproroofingarcadia.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Roof Inspection</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@metalproroofingarcadia.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(833) 642-0267</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Corona CA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Corona CA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-13 11:43 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1083,6 +1083,66 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in Baltimore, MD - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>hvaccontractorbaltimore.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.hvaccontractorbaltimore.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Charles St</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@hvaccontractorbaltimore.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(410) 498-6802</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Baltimore MD</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>heating and cooling company Baltimore MD</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-13 19:12 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1143,6 +1143,122 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Contractor Starter Theme</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>highroadroofing.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://highroadroofing.com/roofing/laramie-wy/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>With Integrity</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@highroadroofing.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(970) 568-7663</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Laramie WY</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>roof replacement Laramie WY</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Baltimore MD HVAC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>baltimoremdhvac.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://baltimoremdhvac.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>konstruck@gmial.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(240) 426-3190</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Baltimore MD</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>HVAC contractor Baltimore MD</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-13 19:15 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1224,7 +1224,6 @@
           <t>https://baltimoremdhvac.com/</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>konstruck@gmial.com</t>
@@ -1254,6 +1253,62 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Irvine, CA | KJC Roofing</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>kjcroofing.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://kjcroofing.com/service-areas/irvine-ca</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@kjcroofing.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>9492280322</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Irvine CA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>80</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>roofing contractor Irvine CA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-13 19:17 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1279,7 +1279,6 @@
           <t>https://kjcroofing.com/service-areas/irvine-ca</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>info@kjcroofing.com</t>
@@ -1309,6 +1308,66 @@
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AC Repair Allentown PA | Same-Day AC Repair in Allentown &amp; the Lehigh Valley</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>acrepairallentown.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://acrepairallentown.com/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Repair Allentown</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ops@acrepairallentown.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(610) 884-6946</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Allentown PA</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>air conditioning repair Allentown PA</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-13 19:18 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1373,6 +1373,62 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Orlandoairconditioningrepair.net</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>orlandoairconditioningrepair.net</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.orlandoairconditioningrepair.net/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>info@orlandoairconditioningrepair.net</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>407-289-0226</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>air conditioning repair Orlando FL</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-13 19:26 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1394,7 +1394,6 @@
           <t>https://www.orlandoairconditioningrepair.net/</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>info@orlandoairconditioningrepair.net</t>
@@ -1424,6 +1423,66 @@
         </is>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Bramwells Cooling &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>bramwellscooling.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://bramwellscooling.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Starting Capacitors</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>bramwellscooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(321) 450-4557</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>86</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>heating and cooling company Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-13 19:29 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-13.xlsx
+++ b/output/leads_2026-10-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1488,6 +1488,62 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ecofficient Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ugoeco.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://ugoeco.com/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>dan@ugoeco.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(517) 862-1020</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>88</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>heating and cooling company Lansing MI</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>